<commit_message>
Refer to the four users as User 1-4 and list Jeremy first
Replace the member IDs with anonymous names (User 1 to User 4) in the
writeup, the spreadsheet, the exported run data, recipes and results.
List Jeremy first among the team members.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Baselines.xlsx
+++ b/Baselines.xlsx
@@ -495,7 +495,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -543,7 +543,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -591,7 +591,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -639,7 +639,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -687,7 +687,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -735,7 +735,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -783,7 +783,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -831,7 +831,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -879,7 +879,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
@@ -927,7 +927,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>jeremyti</t>
+          <t>User 1</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -975,7 +975,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1023,7 +1023,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1071,7 +1071,7 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -1119,7 +1119,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1167,7 +1167,7 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1215,7 +1215,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1263,7 +1263,7 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1311,7 +1311,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1354,7 +1354,7 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1402,7 +1402,7 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>sourajak</t>
+          <t>User 2</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1450,7 +1450,7 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1502,7 +1502,7 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1556,7 +1556,7 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1610,7 +1610,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -1664,7 +1664,7 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -1718,7 +1718,7 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
@@ -1770,7 +1770,7 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1824,7 +1824,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1878,7 +1878,7 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1932,7 +1932,7 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>jgai</t>
+          <t>User 3</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1986,7 +1986,7 @@
     <row r="33">
       <c r="A33" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -2034,7 +2034,7 @@
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
@@ -2083,7 +2083,7 @@
     <row r="35">
       <c r="A35" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
@@ -2131,7 +2131,7 @@
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B36" s="14" t="inlineStr">
@@ -2180,7 +2180,7 @@
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B37" s="14" t="inlineStr">
@@ -2229,7 +2229,7 @@
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B38" s="14" t="inlineStr">
@@ -2277,7 +2277,7 @@
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
@@ -2326,7 +2326,7 @@
     <row r="40">
       <c r="A40" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
@@ -2374,7 +2374,7 @@
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
@@ -2423,7 +2423,7 @@
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>istepka</t>
+          <t>User 4</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
@@ -2480,7 +2480,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E27"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="27.63" customWidth="1" style="16" min="2" max="2"/>
@@ -2495,6 +2495,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -2626,6 +2627,8 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -2661,6 +2664,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="B19" s="6" t="inlineStr">
         <is>

</xml_diff>